<commit_message>
reference_summary와 required_points 보강 후 major_error_criteria 수정
</commit_message>
<xml_diff>
--- a/data/llm_evaluation.xlsx
+++ b/data/llm_evaluation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gyg03\Desktop\MINE\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gyg03\Desktop\project-collection\ai-evaluation-proj\Korean-finance-AI-evaluation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00C3EC35-55A5-4457-90DE-E525216A7442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6582777B-ED0E-4C7E-8B5E-347FE4B31351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{8E6529A6-41F8-41E7-A43C-D6043225C6E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="183">
   <si>
     <t>question_id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -201,38 +201,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t>가장 대표적인 RP형(환매조건부 채권), 발행어음형(발행어음에 투자), 종금형(예금자보호법 적용), MMF</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>ㆍMMW형(펀드 또는 한국증권금융에 위탁) 등이 있다.</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>RP형; 발행어음형; 종금형; MMF</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>ㆍMMW형</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>https://mofe.go.kr/sisa/dictionary/detail?idx=166</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -241,26 +209,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>펀드; 실적배당상품; 시장 금리와 무관; 안정적인 수익률; 자유로운 입출금</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CMA는 계좌; MMF는 펀드; 둘 다 자유로운 입출금; 단기 자금 운용에 적합</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>아님, CMA는 일반 통장의 기능을 가진 계좌이고 MMF는 만기가 짧은 금융 상품에 투자하는 펀드이다. 둘 다 입출금은 자유롭고 단기 자금 운용에 적합</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CMA 유형에 따라 다름, 종금형은 예금자 보호가 되지만, 증권형(MMF, RP등)은 불가능</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CMA 종류에 따라 다름; 종금형만 가능;나머지는 불가능</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>CMA의 수익률은 모든 유형에서 고정되어 있나요?</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -269,31 +217,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>CMA 종류에 따라 다르고, 증권사 CMA의 경우 증권사 마다 상이</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>유형에 따라 상이; 증권사마다 상이</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>https://toss.im/tossfeed/article/toss-cma-interest</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>됨, CMA 중에 종금형만 예금자 보호가 됨</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>예금자 보호 가능</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>예금자 보호 불가, 시장 상황에 따라 원금 전부 또는 일부 손실 위험 있음</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>예금자 보호 불가능; 자금 손실 위험 있음</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -317,14 +241,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>불가능함, 원할 경우 MMF형 CMA로 가입하는 것을 권장</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>불가능</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>CMA에서 발생한 수익에도 세금이 부과되나요?</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -333,10 +249,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>금융소득; 종합소득세</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>RP형 CMA와 MMF형 CMA는 주로 어떤 자산에 투자하나요?</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -357,40 +269,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>CMA: 증권사, 예금자 보호법 적용 불가
-파킹통장: 은행, 예금자 보호법 적용 가능</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CMA는 증권사에서 판매, 예금자 보호 불가;파킹통장은 은행에서, 예금자 보호 가능</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>CMA에 가입하기 전에 상품설명서에 어떤 항목을 우선 확인해야 하나요?</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>예금자 보호 가능 여부, 원금 손실 가능성, 이자율</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>예금자 보호 가능 여부;원금 손실 가능성에 대한 숙지;이자율</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>가능; 수시 입출금 가능</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>가능, 노는 돈을 보관해두고 매일 이자를 받아 대기 자금 관리</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>개인의 상황에 따라 다름, 예금자 보호 여부, 일반 통장과 비슷하게 사용을 원하는지, 원금 손실 감수 여부에 따라 결정해야 한다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>여러 요소 함께 고려 필수;예금자 보호 여부;원금 손실 가능성;입출금과 결제 기능의 필요성</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -815,26 +694,10 @@
     <t>correct</t>
   </si>
   <si>
-    <t>증권사에서 개설할 수 있는 자산관리계좌; 높은 금리; 주식 투자 전 자본 보관 용도; 증권사; 자유로운 입출금</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>자산관리계좌로 수시 입출금보다 상대적으로 높은 금리를 준다, 증권사에서 만들 수 있으며 주식 투자 전 돈을 잠시 보관하는 용도로 활용</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>CMA를 은행의 예·적금 상품으로 설명함; 모든 CMA가 확정금리나 높은 수익을 보장한다고 설명함; 모든 CMA의 원금이 보장되거나 예금자보호 대상이라고 설명함; CMA 자금이 금융상품에 운용되지 않고 단순히 보관된다고 설명함; CMA는 만기 전 출금이 불가능하다고 설명함</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>네 가지를 모두 설명하지 않음;네 가지 중 한 가지라도 이름이나 종류가 다름</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Money Market Funds, 단기금융상품에 집중투자하는 초단기 공사채형 금융상품(단기 금리의 등락이 펀드 수익률에 바로 반영되도록 함), 실적배당상품, 예금자보호 불가</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>펀드라는 점을 설명하지 않음; 장기 자산이라고 설명함; 예금자보호가 된다고 설명함; 고정금리 제공;원금 보장된다고 설명함</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -847,10 +710,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>모든 종류가 예금자 보호가 된다고 설명함; 종금형 외에 다른 종류도 예금자 보호가 된다고 설명함</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>종금형 외에 다른 종류가 예금자보호 대상이라고 설명함</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -863,10 +722,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>세금 부과 대상이 아니라고 설명함; 종합소득세가 아닌 다른 세금으로 안내함</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>RP형을 일반 통장에 자금을 보관한다고 설명함; MMF형을 시중 은행이나 증권사 계좌에 투자한다고 설명함</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -879,10 +734,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>만기 시에만 출금 가능하다고 설명; 단기 상품이 아니라고 설명; MMF가 장기 투자용이라고 설명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>무조건 둘 중 하나가 낫다고 설명; 금리만 고려하면 된다고 설명; 원금 손실 우려 또는 예금자 보호가 되기 때문에 둘 중 아무거나 가입하면 된다고 설명;</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -951,34 +802,14 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>CMA와 MMF가 같지 않다는 점, 세부적인 차이점을 모두 오류없이 설명함</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>종금형 CMA만 가능하다는 점을 오류없이 설명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve"> CMA 유형별로 구분하여 세부적인 사항을 오류없이 설명</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>종금형 CMA는 예금자 보호가 된다는 점을 오류없이 설명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MMF는 예금자 보호 대상이 아니기 때문에 원금 손실 위험이 있다는 점을 오류없이 설명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>MMF는 일반 통장의 기능을 사용할 수 없다는 점, MMF형 CMA를 대체로 사용할 수 있다는 점을 오류없이 설명</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>금융소득이므로 세금 부과 대상이며, 15.4%가 원천징수된다. 2000만원 이상일 경우 종합소득세 합산 신고 해야한다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>partial</t>
   </si>
   <si>
@@ -986,35 +817,280 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>RP형은 증권사가 발행하는 채권에, MMF형은 고객의 자금을 자산 운용사가 만든 펀드에 투자하를 하여 고객에게 나눠주는 실적 배당형 상품이다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RP형은 증권사 채권; MMF형은 자산 운용사가 만든 펀드에 투자</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>RP형과 MMF형 CMA의 투자 대상 차이를 오류없이 설명</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>complete</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CMA와 파킹통장의 세부적인 차이점을 오류없이 설명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CMA를 가입하기 전 가장 중요하게 고려해야 할 사항을 오류없이 설명</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>가능하다는 점, 주의해야 할 점을 오류없이 설명</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MMF를 추천하는 경우에 대한 설명이 상대적으로 적지만, 초보자에게 CMA를 추천하는 이유를 오류없이 설명</t>
+    <r>
+      <t>CMA(Cash Management Account)는 주로 증권사에서 개설하는 자산관리계좌로, 입금한 자금을 RP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㆍMMFㆍMMWㆍ발행어음 등의 단기금융상품에 자동으로 운용하는 구조다. 비교적 자유롭게 입출금할 수 있어 투자 전 대기자금이나 단기 여유 자금 관리에 활용된다. 수익률, 예금자 보호 여부와 출금 조건은 CMA 유형 및 금융회사에 따라 다르다.</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>주로 증권사에서 개설할 수 있는 자산관리계좌; 단기금융상품; 수시 입출금 가능; 유형별 위험과 수익률 차이</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA는 자금 운용 방식에 따라 RP형, 발행어음형, MMF형, MMW형과 예금자보호가 적용되는 종금형 등으로 구분된다. RP형은 환매조건부채권, 발행어음형은 증권사가 발행한 어음, MMF형은 단기금융상품에 투자하는 펀드, MMW형은 한국증권금융 예수금 등의 단기자산으로 운용한다. 모든 금융회사가 모든 유형을 판매하는 것은 아니며, 유형별로 수익 구조와 원금 손실 가능성, 예금자보호 여부가 다르다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>RP형; 발행어음형; 종금형; MMF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㆍMMW형</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; 유형별 운용 방식과 보호 여부가 다름</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>모든 CMA가 같은 자산에 투자한다고 설명; 모든 유형이 예금자보호 대상이라고 설명; 유형에 대한 특징</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Money Market Funds, 여러 투자자의 자금을 모아 국공채, 기업 어음(CP), 양도성예금증서(CD), 콜 등 만기가 짧은 금융상품에 투자하는 펀드다. 운용 실적에 따라 수익이 달라지는 실적배당상품이므로 고정금리나 원금이 보장되지 않는다. 예금자 보호 대상이 아니며, 위험이 비교적 낮은 단기자산에 투자하더라도 시장 상황에 따라 원금 손실이 발생할 수 있다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>펀드; 실적배당상품; 단기 금융 상품에 투자; 고정금리 아님; 예금자보호 불가; 원금 손실 가능성 있음</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>아님. CMA는 고객 자금을 RP</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㆍMMFㆍMMWㆍ발행어음 등에 자동으로 운용할 수 있는 계좌 또는 자금관리 서비스이고, MMF는 단기금융상품에 투자하는 펀드다. 둘 다 단기자금 운용에 활용할 수 있지만, 직접 가입한 MMF는 환매 절차가 필요하고 카드결제ㆍ자동이체 같은 계좌 기능을 자체적으로 제공하지 않는다. CMA의 결제ㆍ출금 기능과 이용 가능 시간은 금융회사와 상품에 따라 다르다.</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA는 계좌 또는 자금관리 서비스; MMF는 펀드; 둘 다 단기자금 운용에 활용 가능; 직접 가입한 MMF는 환매 필요; 계좌 기능의 차이</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>CMA 유형에 따라 다름, RP형</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㆍMMF형ㆍMMW형ㆍ발행어음형 등 일반적인 증권사 CMA 투자상품은 예금자보호 대상이 아니지만, 보호 대상으로 등록된 종금형 CMA는 예금자보호가 적용될 수 있다. 보호 한도는 2025년 9월 1일부터 원금과 소정의 이자를 합해 1인당 금융회사별 최대 1억 원이며,가입 전 상품설명서나 예금자보호 표시를 확인해야 한다.</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA 종류에 따라 다름; 일반적인 증권사 CMA 투자상품은 보호 불가; 보호 대상으로 등록된 종금형 CMA는 보호 가능; 금융회사별 최대 1억원; 상품설명서 확인</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>모든 종류가 예금자 보호가 된다고 설명함; 모든 CMA가 예금자보호 대상이 아니라고 설명하여 종금형 예외를 누락함; 현재 보호 한도를 5천만원이라고 설명함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA 수익률은 모든 유형에서 고정되어 있지 않다. RP형과 발행어음형은 매수 시 금융회사가 고시한 약정수익률이 적용되지만, 새로 입금하거나 재투자할 때 적용되는 수익률은 시장 상황에 따라 바뀔 수 있다. MMF형과 MMW형은 운용 실적 또는 시장금리 등에 따라 수익이 달라지는 실적배당형이다. 적용 수익률은 CMA 유형과 금융회사, 금액 및 기간에 따라 다를 수 있다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>모든 유형에서 고정되지 않음; RP형과 발행어음형은 약정수익률 적용; 재투자 시 수익률 변경 가능; MMF형과 MMW형은 실적에 따라 변동; 금융회사별 차이</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>종금형 CMA는 보호받을 수 있다. 현재 보호 한도는 해당 금융회사의 다른 보호대상 상품과 합산해 1인당 원금과 소정의 이자를 포함한 최대 1억 원이다. 다만 RP형</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㆍMMF형 등 다른 CMA유형까지 같은 보호가 적용되는 것은 아니므로 개별 상품설명서의 예금자보호 표시를 확인해야 한다.</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>종금형 CMA는 보호 가능; 금융회사별 최대 1억원; 같은 금융회사의 다른 보호상품과 합산; 다른 CMA 유형과 구분</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>MMF는 예금자보호 대상이 아니다. 국공채</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㆍCDㆍCP 등 비교적 위험이 낮은 단기금융상품에 분산투자하지만 운용 실적에 따라 수익이 달라지는 펀드이므로 원금이 보장되지 않는다. 시장 상황이다 편입 자산의 가치 변동에 따라 투자 원금의 일부 또는 전부에 손실이 발생할 수 있다.</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예금자보호 불가; 실적배당형 펀드; 원금 보장 불가; 원금 손실 가능</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>직접 가입한 MMF는 펀드이므로 그 자체를 일반 입출금계좌처럼 카드결제</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㆍ자동이체ㆍATM 출금에 사용할 수 없다. 자금을 사용하려면 MMF를 환매해 연결된 결제계좌 등으로 옮겨야 하며, 환매 신청 기간과 판매 회사의 지금 한도에 따라 당일 또는 다음 영업일 이후에 지급될 수 있다. MMF형 CMA는 금융회사가 별도의 결제ㆍ출금 서비스를 제공할 수 있지만, 이용 가능 여부와 조건은 해당 회사의 약관을 확인해야 한다.</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>직접 가입한 MMF는 결제계좌가 아님; 카드결제ㆍ자동이체ㆍATM 출금 직접 이용 불가; 사용하려면 환매 필요; MMF형 CMA와 구분</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA에서 발생한 수익인 상품 유형에 따라 이자소득 또는 배당소득으로 분류되는 금융소득이며, 일반적으로 소득세 14%와 지방소득세1.4%를 합한 15.4%가 원천징수된다. 개인별 연간 이자ㆍ배당소득 합계가 2000만 원 이하이고 국내에서 정상적으로 원천징수됐다면 일반적으로 별도의 종합소득세 합산 신고를 하지 않는다. 과세 대상 금융소득 합계가 2000만 원을 초과하면 금융소득종합과세 대상이 되어 다른 종합소득과 함께 신고해야 한다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA 수익이 모두 비과세라고 설명함; 15.4% 원천징수를 종합소득세와 동일한 개념으로 설명함; 금액과 관계없이 모든 가입자가 종합소득세 신고를 해야 한다고 설명함; 금융소득 2천만원 기준을 원금이나 CMA 잔액 기준이라고 설명함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RP형 CMA는 증권사가 보유한 국채ㆍ지방채ㆍ은행채 등의 채권을 고객에게 매도하고 일정 기간 후 다시 사들이는 환매조건부채권(RP)에 투자한다. MMF형 CMA는 고객 자금을 MMF에 투자하며,해당 펀드는 콜ㆍ국공채ㆍ양도성예금증서(CD)ㆍ기업어음(CP) 등의 단기금융상품으로 운용한다. RP형은 일반적으로 약정수익률 방식이고, MMF형은 운용 실적에 따라 수익이 달라지는 실적배당 방식이다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RP형은 환매조건부채권에 투자; RP의 기초자산은 국채ㆍ지방채ㆍ은행채 등; MMF형은 MMF에 투자; MMF는 콜ㆍ국공채ㆍCDㆍCP 등 단기금융상품에 투자; RP형과 MMF형의 수익 구조 차이</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>파킹통장은 은행이 제공하는 수시입출금식 예금으로, 해당 은행의 다른 보호대상 상품과 합산해 1인당 최대 1억 원까지 예금자보호를 받을 수 있다. CMA는 주로 증권사에서 개설해 RPㆍMMFㆍMMWㆍ발행어음 등에 자금을 운용하는 계좌로, 일반적인 투자형 CMA는 예금자보호 대상이 아니지만 보호 대상으로 등록된 종금형 CMA는 예외가 될 수 있다. 두 상품 모두 단기자금 관리에 활용되지만 수익 구조, 원금 손실 가능성, 결제 기능과 출금 조건이 다르므로 상품설명서를 확인해야 한다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>파킹통장은 은행의 수시입출금식 예금; 파킹통장은 금융회사별 최대 1억원까지 보호 가능;CMA는 단기금융상품에 운용; 원금 손실과 이용 기능 차이</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA 가입 전에는 먼저 RP형ㆍMMF형ㆍ발행어음형 등 운용 유형과 실제 투자 대상을 확인해야 한다. 다음으로 예금자보호 여부와 원금 손실 가능성, 약정수익률인지 실적배당인지, 수익률 변경 조건을 확인해야 한다. 출금 가능 시간과 환매 소요 기간, 카드ㆍ지동이체 지원 여부, 수수료ㆍ세금 및 금융회사의 신용위험도 함께 확인하는 것이 좋다. 표시된 수익률만 보고 상품을 선택해서는 안 된다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA 유형과 운용 대상; 예금자보호 여부; 원금 손실 가능성; 수익률 적용 방식과 변경 조건; 출금ㆍ환매 조건; 결제 기능; 수수료와 세금</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MMF에 투자하는 것은 가능하지만, 한 달 뒤 반드시 사용해야 하는 등록금이라면 무조건 적합하다고 단정할 수 없다. MMF는 예금자 보호 대상이 아니고 원금 손실 가능성이 있으며, 환매 신청 시간이나 판매회사의 지금 한도에 따라 자금 지급이 다음 영업일 이후로 늦어질 수 있다. 원금 손실이나 지급 지연을 감수하기 어려운 자금이라면 예금자보호가 적용되고 즉시 출금 가능한 상품을 함께 비교해야 한다. MMF를 이용한다면 등록금 납부일보다 여유 있게 환매하고 해당 상품의 환매 조건을 확인해야 한다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>투자는 가능하지만 무조건 적합하지 않음; 예금자보호 불가; 원금 손실 가능; 환매대금 지급 지연 가능; 사용 날짜가 정해진 자금은 안정성과 유동성 우선; 환매 조건 확인</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MMF가 원금 보장 상품이므로 등록금을 넣어도 안전하다고 단정함; 납부 직전에도 언제나 즉시 출금할 수 있다고 설명함; 손실 및 환매 지연 가능성을 전혀 고려하지 않고 가입을 권장함</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">투자 경험이 없다는 이유만으로 CMA와 MMF 중 하나가 항상 더 적합하다고 정할 수는 없다. CMA는 계좌 또는 자금관리 서비스이고 MMF는 펀드이며, CMA 안에서 MMF에 자동 투자하는 MMF형 CMA도 있어 두 상품은 완전히 대등한 비교 대상이 아니다. 카드ㆍ이체 등 계좌 기능과 간편한 대기자금 관리를 원한다면 CMA의 기능을 비교할 수 있고, 직접 MMF에 투자하려면 환매 방식과 원금 손실 가능성을 이해해야 한다. 원금 손실을 받아들이기 어렵다면 두 상품을 무조건 선택하기보다 예금자보호가 적용되는 수시입출금 상품도 함께 비교해야 한다. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>개인 상황에 따라 다름; CMA는 계좌 또는 자금관리 서비스; MMF는 펀드; MMF형 CMA도 존재; 필요한 결제ㆍ이체 기능; 원금 손실 감수 여부; 예금자보호 필요성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA와 MMF가 같지 않다는 점, 세부적인 차이점을 거의 오류없이 설명했지만 MMF는 환매가 반드시 필요하다는 점 설명 누락</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>need_revision</t>
+  </si>
+  <si>
+    <t>종금형 CMA만 가능하다는 점은 맞지만, 예금자보호법 기준 2025년 9월 1일 이후로는 1인당 최대 1억원까지 보호되므로 부분적인 오류</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>minor_error</t>
+  </si>
+  <si>
+    <t>종금형 CMA는 예금자 보호가 된다는 점은 맞지만 1인당 최고 5천만원이 아닌 1억원까지 보호됨(지난 정보 업데이트 필요)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MMF는 예금자 보호 대상이 아니라는 점은 맞지만 1인단 최고 5천만원이라는 점은 오류, MMF가 실적배당형 상품이라는 점 누락</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>금융소득; 유형에 따라 이자소득 또는 배당소득; 일반적으로 15.4% 원천징수; 연간 금융소득 2천만원 기준; 원천징수와 종합과제의 구분</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>partial</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA와 파킹통장의 세부적인 차이점은 오류없이 설명했지만 예금자보호는 1인당 최대 5천만원이 아닌 1억 원까지 가능</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CMA를 가입하기 전 가장 중요하게 고려해야 할 사항을 오류없이 설명했지만 1인당 최대 5천만원이라는 예금자보호에 관한 설명이 오류</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MMF를 추천하는 경우에 대한 설명이 상대적으로 적으며 예금자보호에 관련된 설명 없음, 초보자에게 CMA를 추천하는 이유를 오류없이 설명</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1121,9 +1197,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1133,6 +1206,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1166,42 +1242,9 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
           <bgColor theme="9" tint="0.59999389629810485"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1240,6 +1283,39 @@
       </fill>
       <alignment vertical="center" textRotation="0" wrapText="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1254,7 +1330,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F824F088-8F03-4AD2-A736-626536A353C7}" name="표1" displayName="표1" ref="B1:I16" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F824F088-8F03-4AD2-A736-626536A353C7}" name="표1" displayName="표1" ref="B1:I16" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
   <autoFilter ref="B1:I16" xr:uid="{F824F088-8F03-4AD2-A736-626536A353C7}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1266,21 +1342,21 @@
     <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{9CE8D845-33AA-43B9-B765-A7A55E11AB3C}" name="question_id" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{96F77B20-A6A8-4EE3-95DF-4EEA2B98C840}" name="query_type" dataDxfId="23"/>
-    <tableColumn id="3" xr3:uid="{572AE9E3-2226-4139-83BE-6E1ECAE9FF6F}" name="question" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{2AB870EA-B725-4924-B6E3-71C21C5D778D}" name="reference_url" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{A9186594-909D-4690-B88E-5E5D260928D3}" name="checked_at" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{2CCDED83-45BF-4007-AAAC-22FF9A60F028}" name="reference_summary" dataDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{D8720B7C-9BC0-4295-9D05-DCC0BA9D4F44}" name="major_error_criteria" dataDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{F6977487-A6B1-45F3-B42A-877A2562B7EE}" name="required_points" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{9CE8D845-33AA-43B9-B765-A7A55E11AB3C}" name="question_id" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{96F77B20-A6A8-4EE3-95DF-4EEA2B98C840}" name="query_type" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{572AE9E3-2226-4139-83BE-6E1ECAE9FF6F}" name="question" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{2AB870EA-B725-4924-B6E3-71C21C5D778D}" name="reference_url" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{A9186594-909D-4690-B88E-5E5D260928D3}" name="checked_at" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{2CCDED83-45BF-4007-AAAC-22FF9A60F028}" name="reference_summary" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{D8720B7C-9BC0-4295-9D05-DCC0BA9D4F44}" name="major_error_criteria" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{F6977487-A6B1-45F3-B42A-877A2562B7EE}" name="required_points" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium16" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{73E9684D-1207-4205-B8B4-26D368E340F2}" name="표2" displayName="표2" ref="A1:F16" totalsRowShown="0" headerRowDxfId="15" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{73E9684D-1207-4205-B8B4-26D368E340F2}" name="표2" displayName="표2" ref="A1:F16" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
   <autoFilter ref="A1:F16" xr:uid="{73E9684D-1207-4205-B8B4-26D368E340F2}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1302,7 +1378,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A09A038D-63EC-4F00-8471-614B8DEBC74A}" name="표3" displayName="표3" ref="A1:G16" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A09A038D-63EC-4F00-8471-614B8DEBC74A}" name="표3" displayName="표3" ref="A1:G16" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
   <autoFilter ref="A1:G16" xr:uid="{A09A038D-63EC-4F00-8471-614B8DEBC74A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -1313,13 +1389,13 @@
     <filterColumn colId="6" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{4F8152B0-027C-4A0D-9A3C-46BD7423928B}" name="annotation_id" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{C4F890A6-ABD3-4535-A71A-C7AE4C3F85E1}" name="response_id" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{AB966220-A78C-4FBC-858D-38B27296116B}" name="question_id" dataDxfId="12"/>
-    <tableColumn id="4" xr3:uid="{AD43F1FC-7C1E-4A33-8FBF-17D3C765870E}" name="accuracy" dataDxfId="11"/>
-    <tableColumn id="5" xr3:uid="{A9374898-350D-44EC-AA40-11F66142A1A8}" name="completeness" dataDxfId="10"/>
-    <tableColumn id="6" xr3:uid="{E39A8687-2B8A-47F1-9719-CE73F0C19944}" name="final_label" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{FFBD66D0-27B4-497C-9EE0-0934541D0303}" name="annotation_note" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{4F8152B0-027C-4A0D-9A3C-46BD7423928B}" name="annotation_id" dataDxfId="24"/>
+    <tableColumn id="2" xr3:uid="{C4F890A6-ABD3-4535-A71A-C7AE4C3F85E1}" name="response_id" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{AB966220-A78C-4FBC-858D-38B27296116B}" name="question_id" dataDxfId="22"/>
+    <tableColumn id="4" xr3:uid="{AD43F1FC-7C1E-4A33-8FBF-17D3C765870E}" name="accuracy" dataDxfId="21"/>
+    <tableColumn id="5" xr3:uid="{A9374898-350D-44EC-AA40-11F66142A1A8}" name="completeness" dataDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{E39A8687-2B8A-47F1-9719-CE73F0C19944}" name="final_label" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{FFBD66D0-27B4-497C-9EE0-0934541D0303}" name="annotation_note" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1682,8 +1758,8 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="121.8" x14ac:dyDescent="0.4">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="1:9" ht="139.19999999999999" x14ac:dyDescent="0.4">
+      <c r="A2" s="11" t="s">
         <v>30</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1700,17 +1776,17 @@
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="1" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="69.599999999999994" x14ac:dyDescent="0.4">
-      <c r="A3" s="7"/>
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="156.6" x14ac:dyDescent="0.4">
+      <c r="A3" s="11"/>
       <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
@@ -1725,17 +1801,17 @@
       </c>
       <c r="F3" s="4"/>
       <c r="G3" s="1" t="s">
-        <v>43</v>
+        <v>141</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="69.599999999999994" x14ac:dyDescent="0.4">
-      <c r="A4" s="7"/>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="139.19999999999999" x14ac:dyDescent="0.4">
+      <c r="A4" s="11"/>
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1746,21 +1822,21 @@
         <v>21</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="1" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>131</v>
+        <v>103</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="87" x14ac:dyDescent="0.4">
-      <c r="A5" s="7"/>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="156.6" x14ac:dyDescent="0.4">
+      <c r="A5" s="11"/>
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
@@ -1771,21 +1847,21 @@
         <v>22</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="1" t="s">
-        <v>49</v>
+        <v>146</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>132</v>
+        <v>104</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="52.2" x14ac:dyDescent="0.4">
-      <c r="A6" s="7" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="139.19999999999999" x14ac:dyDescent="0.4">
+      <c r="A6" s="11" t="s">
         <v>27</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1802,17 +1878,17 @@
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="1" t="s">
-        <v>50</v>
+        <v>148</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="104.4" x14ac:dyDescent="0.4">
-      <c r="A7" s="7"/>
+        <v>149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="139.19999999999999" x14ac:dyDescent="0.4">
+      <c r="A7" s="11"/>
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
@@ -1820,24 +1896,24 @@
         <v>34</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="1" t="s">
-        <v>54</v>
+        <v>151</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>133</v>
+        <v>105</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="69.599999999999994" x14ac:dyDescent="0.4">
-      <c r="A8" s="7"/>
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="121.8" x14ac:dyDescent="0.4">
+      <c r="A8" s="11"/>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
@@ -1848,21 +1924,21 @@
         <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="1" t="s">
-        <v>57</v>
+        <v>153</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>135</v>
+        <v>106</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="52.2" x14ac:dyDescent="0.4">
-      <c r="A9" s="7"/>
+        <v>154</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="121.8" x14ac:dyDescent="0.4">
+      <c r="A9" s="11"/>
       <c r="B9" s="1" t="s">
         <v>11</v>
       </c>
@@ -1873,20 +1949,20 @@
         <v>25</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="1" t="s">
-        <v>59</v>
+        <v>155</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>136</v>
+        <v>107</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="104.4" x14ac:dyDescent="0.4">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="174" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>29</v>
       </c>
@@ -1897,23 +1973,23 @@
         <v>34</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="F10" s="4"/>
       <c r="G10" s="1" t="s">
-        <v>63</v>
+        <v>157</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>137</v>
+        <v>108</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="78" customHeight="1" x14ac:dyDescent="0.4">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="174" x14ac:dyDescent="0.4">
       <c r="B11" s="1" t="s">
         <v>13</v>
       </c>
@@ -1921,20 +1997,20 @@
         <v>34</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="F11" s="4"/>
       <c r="G11" s="1" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>138</v>
+        <v>160</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>67</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:9" s="1" customFormat="1" ht="348" x14ac:dyDescent="0.4">
@@ -1945,24 +2021,24 @@
         <v>33</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="F12" s="4"/>
       <c r="G12" s="1" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="87" x14ac:dyDescent="0.4">
-      <c r="A13" s="7" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="191.4" x14ac:dyDescent="0.4">
+      <c r="A13" s="11" t="s">
         <v>28</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -1975,21 +2051,21 @@
         <v>26</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="1" t="s">
-        <v>73</v>
+        <v>163</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>140</v>
+        <v>110</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="52.2" x14ac:dyDescent="0.4">
-      <c r="A14" s="7"/>
+        <v>164</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="156.6" x14ac:dyDescent="0.4">
+      <c r="A14" s="11"/>
       <c r="B14" s="1" t="s">
         <v>16</v>
       </c>
@@ -1997,24 +2073,24 @@
         <v>35</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>40</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="1" t="s">
-        <v>76</v>
+        <v>165</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="52.2" x14ac:dyDescent="0.4">
-      <c r="A15" s="7"/>
+        <v>166</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="191.4" x14ac:dyDescent="0.4">
+      <c r="A15" s="11"/>
       <c r="B15" s="1" t="s">
         <v>17</v>
       </c>
@@ -2022,24 +2098,24 @@
         <v>35</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="E15" s="5" t="s">
         <v>41</v>
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="1" t="s">
-        <v>79</v>
+        <v>167</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>142</v>
+        <v>169</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="69.599999999999994" x14ac:dyDescent="0.4">
-      <c r="A16" s="7"/>
+        <v>168</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="208.8" x14ac:dyDescent="0.4">
+      <c r="A16" s="11"/>
       <c r="B16" s="1" t="s">
         <v>18</v>
       </c>
@@ -2047,17 +2123,17 @@
         <v>35</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="1" t="s">
-        <v>80</v>
+        <v>170</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>143</v>
+        <v>112</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>81</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -2104,297 +2180,297 @@
     <col min="2" max="2" width="10.796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.09765625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="60.796875" style="8" customWidth="1"/>
+    <col min="5" max="5" width="60.796875" style="7" customWidth="1"/>
     <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A1" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" s="10" t="s">
+      <c r="A1" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="D1" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>86</v>
+      <c r="C1" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="408.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>103</v>
+        <v>81</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>79</v>
       </c>
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:6" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>106</v>
+        <v>81</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>82</v>
       </c>
       <c r="F3" s="1"/>
     </row>
     <row r="4" spans="1:6" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>107</v>
+        <v>81</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>83</v>
       </c>
       <c r="F4" s="1"/>
     </row>
     <row r="5" spans="1:6" ht="348" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>108</v>
+        <v>81</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>84</v>
       </c>
       <c r="F5" s="1"/>
     </row>
     <row r="6" spans="1:6" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
-        <v>91</v>
+        <v>67</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>109</v>
+        <v>81</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>85</v>
       </c>
       <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:6" ht="313.2" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>110</v>
+        <v>81</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>86</v>
       </c>
       <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:6" ht="226.2" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>111</v>
+        <v>81</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>87</v>
       </c>
       <c r="F8" s="1"/>
     </row>
     <row r="9" spans="1:6" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>112</v>
+        <v>81</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>88</v>
       </c>
       <c r="F9" s="1"/>
     </row>
     <row r="10" spans="1:6" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>113</v>
+        <v>81</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>89</v>
       </c>
       <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" ht="226.2" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>114</v>
+        <v>81</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>90</v>
       </c>
       <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:6" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E12" s="8" t="s">
-        <v>115</v>
+        <v>81</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>91</v>
       </c>
       <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" ht="365.4" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>116</v>
+        <v>81</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>92</v>
       </c>
       <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:6" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>117</v>
+        <v>81</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>93</v>
       </c>
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E15" s="8" t="s">
-        <v>118</v>
+        <v>81</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>94</v>
       </c>
       <c r="F15" s="1"/>
     </row>
     <row r="16" spans="1:6" ht="409.6" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>104</v>
+        <v>80</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>119</v>
+        <v>81</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>95</v>
       </c>
       <c r="F16" s="1"/>
     </row>
@@ -2415,378 +2491,378 @@
     <col min="1" max="1" width="12.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.19921875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.8984375" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
     <col min="5" max="5" width="12.8984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="6" max="6" width="11.796875" customWidth="1"/>
     <col min="7" max="7" width="32.59765625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.4">
-      <c r="A1" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="C1" s="11" t="s">
+      <c r="A1" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="F1" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="G1" s="11" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="69.599999999999994" x14ac:dyDescent="0.4">
+      <c r="D1" s="10" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
-        <v>144</v>
+        <v>113</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>87</v>
+        <v>63</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>161</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
-        <v>145</v>
+        <v>114</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>162</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
-        <v>146</v>
+        <v>115</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
-        <v>147</v>
+        <v>116</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
-        <v>148</v>
+        <v>117</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>91</v>
+        <v>67</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>125</v>
+        <v>175</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>125</v>
+        <v>175</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="52.2" x14ac:dyDescent="0.4">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
-        <v>151</v>
+        <v>120</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>125</v>
+        <v>175</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="52.2" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
-        <v>152</v>
+        <v>121</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>95</v>
+        <v>71</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>169</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
-        <v>153</v>
+        <v>122</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>172</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
-        <v>154</v>
+        <v>123</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
-        <v>155</v>
+        <v>124</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="69.599999999999994" x14ac:dyDescent="0.4">
+      <c r="A14" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="E13" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
-      <c r="A14" s="1" t="s">
-        <v>156</v>
-      </c>
       <c r="B14" s="1" t="s">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>125</v>
+        <v>175</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>159</v>
+        <v>135</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="34.799999999999997" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
-        <v>157</v>
+        <v>126</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>159</v>
+        <v>128</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>160</v>
+        <v>129</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="52.2" x14ac:dyDescent="0.4">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="69.599999999999994" x14ac:dyDescent="0.4">
       <c r="A16" s="1" t="s">
-        <v>158</v>
+        <v>127</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>171</v>
+        <v>135</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.4">

</xml_diff>